<commit_message>
#7 BOM Updated with L2 (VLS5045EX-3R3N)
</commit_message>
<xml_diff>
--- a/Design-Files_v1.3/Deliverables/BOM/Client_BOM-v1.3.xlsx
+++ b/Design-Files_v1.3/Deliverables/BOM/Client_BOM-v1.3.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\antonmeyer-pcbtroubleshoot\Design-Files_v1.3\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\GitHub\antonmeyer-pcbtroubleshoot\Design-Files_v1.3\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75F55CB-E01E-415B-B079-64666E3665A5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -232,9 +233,6 @@
     <t>TSW SMD-6*6*5</t>
   </si>
   <si>
-    <t>IND_CLF7045T-3R3N-D</t>
-  </si>
-  <si>
     <t>LED 0603B</t>
   </si>
   <si>
@@ -367,9 +365,6 @@
     <t>6*6*5</t>
   </si>
   <si>
-    <t>CLF7045T-3R3N-D</t>
-  </si>
-  <si>
     <t>GREEN</t>
   </si>
   <si>
@@ -416,12 +411,18 @@
   </si>
   <si>
     <t>Value</t>
+  </si>
+  <si>
+    <t>VLS5045EX-3R3N</t>
+  </si>
+  <si>
+    <t>IND_VLS5045EX-3R3N</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -906,7 +907,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -954,19 +955,19 @@
         <v>62</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -986,7 +987,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="7"/>
       <c r="I3" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J3" s="7">
         <v>10</v>
@@ -1010,7 +1011,7 @@
       <c r="G4" s="10"/>
       <c r="H4" s="9"/>
       <c r="I4" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1034,7 +1035,7 @@
       <c r="G5" s="8"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1058,7 +1059,7 @@
       <c r="G6" s="10"/>
       <c r="H6" s="9"/>
       <c r="I6" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J6" s="9">
         <v>2</v>
@@ -1082,7 +1083,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1107,10 +1108,10 @@
       </c>
       <c r="G8" s="10"/>
       <c r="H8" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1135,10 +1136,10 @@
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1162,7 +1163,7 @@
       <c r="G10" s="10"/>
       <c r="H10" s="9"/>
       <c r="I10" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1187,10 +1188,10 @@
       </c>
       <c r="G11" s="8"/>
       <c r="H11" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1214,7 +1215,7 @@
       <c r="G12" s="10"/>
       <c r="H12" s="9"/>
       <c r="I12" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1238,7 +1239,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="7"/>
       <c r="I13" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J13" s="7">
         <v>3</v>
@@ -1261,10 +1262,10 @@
       </c>
       <c r="G14" s="10"/>
       <c r="H14" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1290,7 +1291,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="7"/>
       <c r="I15" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1316,7 +1317,7 @@
       <c r="G16" s="10"/>
       <c r="H16" s="9"/>
       <c r="I16" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1342,7 +1343,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="7"/>
       <c r="I17" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1361,12 +1362,12 @@
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="9" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="G18" s="10"/>
       <c r="H18" s="9"/>
       <c r="I18" s="10" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1387,12 +1388,12 @@
         <v>49</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="7"/>
       <c r="I19" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1411,14 +1412,14 @@
       </c>
       <c r="E20" s="10"/>
       <c r="F20" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G20" s="10"/>
       <c r="H20" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J20" s="9">
         <v>2</v>
@@ -1437,12 +1438,12 @@
       </c>
       <c r="E21" s="8"/>
       <c r="F21" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="7"/>
       <c r="I21" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1461,12 +1462,12 @@
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G22" s="10"/>
       <c r="H22" s="9"/>
       <c r="I22" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J22" s="9">
         <v>4</v>
@@ -1485,12 +1486,12 @@
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G23" s="8"/>
       <c r="H23" s="7"/>
       <c r="I23" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1513,16 +1514,16 @@
         <v>50</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
@@ -1543,16 +1544,16 @@
         <v>51</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="J25" s="7">
         <v>4</v>
@@ -1575,16 +1576,16 @@
         <v>52</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J26" s="9">
         <v>4</v>
@@ -1603,12 +1604,12 @@
       </c>
       <c r="E27" s="8"/>
       <c r="F27" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="7"/>
       <c r="I27" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1631,16 +1632,16 @@
         <v>53</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -1661,12 +1662,12 @@
         <v>54</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="7"/>
       <c r="I29" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -1689,16 +1690,16 @@
         <v>55</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -1721,16 +1722,16 @@
         <v>56</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -1751,12 +1752,12 @@
         <v>57</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G32" s="10"/>
       <c r="H32" s="9"/>
       <c r="I32" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -1779,16 +1780,16 @@
         <v>58</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -1809,12 +1810,12 @@
         <v>59</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G34" s="10"/>
       <c r="H34" s="9"/>
       <c r="I34" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -1833,12 +1834,12 @@
       </c>
       <c r="E35" s="8"/>
       <c r="F35" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="7"/>
       <c r="I35" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -1861,16 +1862,16 @@
         <v>60</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -1893,16 +1894,16 @@
         <v>61</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>

</xml_diff>

<commit_message>
#7 U6 Changes in SCH and PCB
</commit_message>
<xml_diff>
--- a/Design-Files_v1.3/Deliverables/BOM/Client_BOM-v1.3.xlsx
+++ b/Design-Files_v1.3/Deliverables/BOM/Client_BOM-v1.3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\GitHub\antonmeyer-pcbtroubleshoot\Design-Files_v1.3\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75F55CB-E01E-415B-B079-64666E3665A5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{039D3766-3B45-4F9C-8D7D-F2DE6E3CE514}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="131">
   <si>
     <t>#</t>
   </si>
@@ -263,9 +263,6 @@
     <t>SK6812 SIDE-A</t>
   </si>
   <si>
-    <t>HDR-TH_5P-P1.27-V-M</t>
-  </si>
-  <si>
     <t>SPL06-001</t>
   </si>
   <si>
@@ -401,9 +398,6 @@
     <t>ULN2003</t>
   </si>
   <si>
-    <t>HLK-LD2410B</t>
-  </si>
-  <si>
     <t>Quantity</t>
   </si>
   <si>
@@ -417,6 +411,9 @@
   </si>
   <si>
     <t>IND_VLS5045EX-3R3N</t>
+  </si>
+  <si>
+    <t>ZX-MX1.25-5PZZ</t>
   </si>
 </sst>
 </file>
@@ -955,19 +952,19 @@
         <v>62</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -987,7 +984,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="7"/>
       <c r="I3" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J3" s="7">
         <v>10</v>
@@ -1011,7 +1008,7 @@
       <c r="G4" s="10"/>
       <c r="H4" s="9"/>
       <c r="I4" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1035,7 +1032,7 @@
       <c r="G5" s="8"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1059,7 +1056,7 @@
       <c r="G6" s="10"/>
       <c r="H6" s="9"/>
       <c r="I6" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J6" s="9">
         <v>2</v>
@@ -1083,7 +1080,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1108,10 +1105,10 @@
       </c>
       <c r="G8" s="10"/>
       <c r="H8" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1136,10 +1133,10 @@
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1163,7 +1160,7 @@
       <c r="G10" s="10"/>
       <c r="H10" s="9"/>
       <c r="I10" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1188,10 +1185,10 @@
       </c>
       <c r="G11" s="8"/>
       <c r="H11" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1215,7 +1212,7 @@
       <c r="G12" s="10"/>
       <c r="H12" s="9"/>
       <c r="I12" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1239,7 +1236,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="7"/>
       <c r="I13" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J13" s="7">
         <v>3</v>
@@ -1262,10 +1259,10 @@
       </c>
       <c r="G14" s="10"/>
       <c r="H14" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1291,7 +1288,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="7"/>
       <c r="I15" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1317,7 +1314,7 @@
       <c r="G16" s="10"/>
       <c r="H16" s="9"/>
       <c r="I16" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1343,7 +1340,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="7"/>
       <c r="I17" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1362,12 +1359,12 @@
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G18" s="10"/>
       <c r="H18" s="9"/>
       <c r="I18" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1393,7 +1390,7 @@
       <c r="G19" s="8"/>
       <c r="H19" s="7"/>
       <c r="I19" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1416,10 +1413,10 @@
       </c>
       <c r="G20" s="10"/>
       <c r="H20" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J20" s="9">
         <v>2</v>
@@ -1443,7 +1440,7 @@
       <c r="G21" s="8"/>
       <c r="H21" s="7"/>
       <c r="I21" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1467,7 +1464,7 @@
       <c r="G22" s="10"/>
       <c r="H22" s="9"/>
       <c r="I22" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J22" s="9">
         <v>4</v>
@@ -1491,7 +1488,7 @@
       <c r="G23" s="8"/>
       <c r="H23" s="7"/>
       <c r="I23" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1517,13 +1514,13 @@
         <v>73</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
@@ -1547,13 +1544,13 @@
         <v>73</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J25" s="7">
         <v>4</v>
@@ -1579,13 +1576,13 @@
         <v>73</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J26" s="9">
         <v>4</v>
@@ -1609,7 +1606,7 @@
       <c r="G27" s="8"/>
       <c r="H27" s="7"/>
       <c r="I27" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1635,13 +1632,13 @@
         <v>73</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -1667,7 +1664,7 @@
       <c r="G29" s="8"/>
       <c r="H29" s="7"/>
       <c r="I29" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -1696,7 +1693,7 @@
         <v>75</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I30" s="10" t="s">
         <v>75</v>
@@ -1725,13 +1722,13 @@
         <v>76</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -1757,7 +1754,7 @@
       <c r="G32" s="10"/>
       <c r="H32" s="9"/>
       <c r="I32" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -1783,13 +1780,13 @@
         <v>78</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -1834,12 +1831,12 @@
       </c>
       <c r="E35" s="8"/>
       <c r="F35" s="7" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="7"/>
       <c r="I35" s="8" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -1862,16 +1859,16 @@
         <v>60</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -1894,16 +1891,16 @@
         <v>61</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>

</xml_diff>